<commit_message>
add energy demand of transport for post processing calculations
</commit_message>
<xml_diff>
--- a/Spine_Projects/01_input_data/04_iaee_2026/02_input_data_raw/Chile_Mining_PtX_Assumptions_clean.xlsx
+++ b/Spine_Projects/01_input_data/04_iaee_2026/02_input_data_raw/Chile_Mining_PtX_Assumptions_clean.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\01_input_data\04_iaee_2026\02_input_data_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{237EEF1D-F392-44F9-B0AA-583EB69A50A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1728C29F-5954-4000-A1B8-DFBB50DD4E39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,9 +16,10 @@
     <sheet name="Input Parameters" sheetId="6" r:id="rId1"/>
     <sheet name="Parameters" sheetId="1" r:id="rId2"/>
     <sheet name="Demand Calculations" sheetId="2" r:id="rId3"/>
-    <sheet name="CO2 Calculations" sheetId="3" r:id="rId4"/>
-    <sheet name="Scenarios &amp; Assumptions" sheetId="4" r:id="rId5"/>
-    <sheet name="Sources" sheetId="5" r:id="rId6"/>
+    <sheet name="Transportation Calculations" sheetId="7" r:id="rId4"/>
+    <sheet name="CO2 Calculations" sheetId="3" r:id="rId5"/>
+    <sheet name="Scenarios &amp; Assumptions" sheetId="4" r:id="rId6"/>
+    <sheet name="Sources" sheetId="5" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="304">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="758" uniqueCount="342">
   <si>
     <t>Final model values used across the workbook; calculations are shown on the following sheets.</t>
   </si>
@@ -950,15 +951,130 @@
   </si>
   <si>
     <t>CO2 cost</t>
+  </si>
+  <si>
+    <t>energy demand for transport methanol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Methanol truck transport </t>
+  </si>
+  <si>
+    <t>Transport Calculations and Assumptions</t>
+  </si>
+  <si>
+    <t>demand for transporting ammonia or methanl via truck</t>
+  </si>
+  <si>
+    <t>energy demand of trucks</t>
+  </si>
+  <si>
+    <t>MJ/km/t</t>
+  </si>
+  <si>
+    <t>S9</t>
+  </si>
+  <si>
+    <t>CSEI Report</t>
+  </si>
+  <si>
+    <t>Range</t>
+  </si>
+  <si>
+    <t>1 to 5</t>
+  </si>
+  <si>
+    <t>demand for uphill transportation demand for transport methanol</t>
+  </si>
+  <si>
+    <t>assumption</t>
+  </si>
+  <si>
+    <t>demand for downhil transportation demand for transport methanol</t>
+  </si>
+  <si>
+    <t>MWh/km/MWh methanol</t>
+  </si>
+  <si>
+    <t>km</t>
+  </si>
+  <si>
+    <t>Distance</t>
+  </si>
+  <si>
+    <t>transport distance Coloso to Escondida</t>
+  </si>
+  <si>
+    <t xml:space="preserve">transport distance Coloso to intersection </t>
+  </si>
+  <si>
+    <t>transport distance escondida to intersection</t>
+  </si>
+  <si>
+    <t>energy demand from escondida to port</t>
+  </si>
+  <si>
+    <t>transport demand in case of export methanol and production at the mine</t>
+  </si>
+  <si>
+    <t>energy demand from intersection to port</t>
+  </si>
+  <si>
+    <t>transport demand in case of export methanol and production at the intersection</t>
+  </si>
+  <si>
+    <t>transport demand in case of transport methanol to the mine and production at the intersection</t>
+  </si>
+  <si>
+    <t>energy demand from port to escondida</t>
+  </si>
+  <si>
+    <t>energy demand from intersection to escondida</t>
+  </si>
+  <si>
+    <t>transport demand in case of transport methanol to the mine and production at the port</t>
+  </si>
+  <si>
+    <t>Ammonia transport demand</t>
+  </si>
+  <si>
+    <t>fixed value</t>
+  </si>
+  <si>
+    <t>MWh/km/MWh ammonia</t>
+  </si>
+  <si>
+    <t>demand for  transportation demand for transport ammonia</t>
+  </si>
+  <si>
+    <t>energy demand for transport ammonia</t>
+  </si>
+  <si>
+    <t>transport demand</t>
+  </si>
+  <si>
+    <t>used to calculate cost based on LCOE results</t>
+  </si>
+  <si>
+    <t>MWh/MWh ammonia</t>
+  </si>
+  <si>
+    <t>MWh/MWh methanol</t>
+  </si>
+  <si>
+    <t>energy demand from inters. to port</t>
+  </si>
+  <si>
+    <t>energy demand from inters. to escondida</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="#,##0.0000"/>
+    <numFmt numFmtId="167" formatCode="#,##0.000000"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -1172,7 +1288,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1237,6 +1353,10 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1249,23 +1369,16 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1434,36 +1547,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8B2ECBF-0ED5-47F2-B014-0A48C60BF7C3}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="11.08203125" customWidth="1"/>
-    <col min="2" max="2" width="27" customWidth="1"/>
+    <col min="2" max="2" width="34.58203125" customWidth="1"/>
     <col min="3" max="3" width="11.1640625" customWidth="1"/>
-    <col min="4" max="4" width="9.6640625" customWidth="1"/>
+    <col min="4" max="4" width="18.25" customWidth="1"/>
     <col min="5" max="5" width="20.75" customWidth="1"/>
     <col min="6" max="6" width="41.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="24" t="s">
         <v>288</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="24"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="26"/>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
@@ -1513,7 +1626,7 @@
       <c r="B6" s="6" t="s">
         <v>292</v>
       </c>
-      <c r="C6" s="31">
+      <c r="C6" s="23">
         <f>'Demand Calculations'!B22</f>
         <v>3645833.3333333335</v>
       </c>
@@ -1534,7 +1647,7 @@
       <c r="B7" t="s">
         <v>294</v>
       </c>
-      <c r="C7" s="31">
+      <c r="C7" s="23">
         <f>'CO2 Calculations'!B31</f>
         <v>591118.81751083327</v>
       </c>
@@ -1548,7 +1661,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="28">
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>301</v>
       </c>
@@ -1569,7 +1682,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="28">
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>301</v>
       </c>
@@ -1590,7 +1703,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="28">
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
         <v>301</v>
       </c>
@@ -1609,6 +1722,174 @@
       </c>
       <c r="F10" t="s">
         <v>302</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" t="s">
+        <v>301</v>
+      </c>
+      <c r="B11" s="29" t="s">
+        <v>323</v>
+      </c>
+      <c r="C11">
+        <f>'Transportation Calculations'!B10</f>
+        <v>1.7085427135678392E-2</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="E11" t="s">
+        <v>336</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" t="s">
+        <v>301</v>
+      </c>
+      <c r="B12" s="29" t="s">
+        <v>340</v>
+      </c>
+      <c r="C12">
+        <f>'Transportation Calculations'!B11</f>
+        <v>1.0552763819095477E-2</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="E12" t="s">
+        <v>336</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" t="s">
+        <v>301</v>
+      </c>
+      <c r="B13" s="29" t="s">
+        <v>341</v>
+      </c>
+      <c r="C13">
+        <f>'Transportation Calculations'!B12</f>
+        <v>1.6331658291457288E-2</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="E13" t="s">
+        <v>336</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" t="s">
+        <v>301</v>
+      </c>
+      <c r="B14" s="29" t="s">
+        <v>328</v>
+      </c>
+      <c r="C14">
+        <f>'Transportation Calculations'!B13</f>
+        <v>4.2713567839195984E-2</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="E14" t="s">
+        <v>336</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" t="s">
+        <v>301</v>
+      </c>
+      <c r="B15" s="29" t="s">
+        <v>323</v>
+      </c>
+      <c r="C15">
+        <f>'Transportation Calculations'!B18</f>
+        <v>5.288888888888889E-3</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>338</v>
+      </c>
+      <c r="E15" t="s">
+        <v>336</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" t="s">
+        <v>301</v>
+      </c>
+      <c r="B16" s="29" t="s">
+        <v>340</v>
+      </c>
+      <c r="C16">
+        <f>'Transportation Calculations'!B19</f>
+        <v>3.2666666666666664E-3</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>338</v>
+      </c>
+      <c r="E16" t="s">
+        <v>336</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" t="s">
+        <v>301</v>
+      </c>
+      <c r="B17" s="29" t="s">
+        <v>341</v>
+      </c>
+      <c r="C17">
+        <f>'Transportation Calculations'!B20</f>
+        <v>2.0222222222222221E-3</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>338</v>
+      </c>
+      <c r="E17" t="s">
+        <v>336</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" t="s">
+        <v>301</v>
+      </c>
+      <c r="B18" s="29" t="s">
+        <v>328</v>
+      </c>
+      <c r="C18">
+        <f>'Transportation Calculations'!B21</f>
+        <v>5.288888888888889E-3</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>338</v>
+      </c>
+      <c r="E18" t="s">
+        <v>336</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>337</v>
       </c>
     </row>
   </sheetData>
@@ -1622,7 +1903,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="13.75" customWidth="1"/>
@@ -1635,26 +1916,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="19" customHeight="1">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="24" t="s">
         <v>288</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="24"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="26"/>
     </row>
     <row r="2" spans="1:7" ht="12" customHeight="1">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
     </row>
     <row r="4" spans="1:7" ht="11" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -2229,6 +2510,48 @@
       </c>
       <c r="G28" s="12" t="s">
         <v>85</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="28">
+      <c r="A29" s="28" t="s">
+        <v>319</v>
+      </c>
+      <c r="B29" s="29" t="s">
+        <v>320</v>
+      </c>
+      <c r="C29">
+        <v>170</v>
+      </c>
+      <c r="D29" s="29" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="28">
+      <c r="A30" s="28" t="s">
+        <v>319</v>
+      </c>
+      <c r="B30" s="29" t="s">
+        <v>321</v>
+      </c>
+      <c r="C30">
+        <v>105</v>
+      </c>
+      <c r="D30" s="29" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" s="28" t="s">
+        <v>319</v>
+      </c>
+      <c r="B31" t="s">
+        <v>322</v>
+      </c>
+      <c r="C31">
+        <v>65</v>
+      </c>
+      <c r="D31" s="29" t="s">
+        <v>318</v>
       </c>
     </row>
   </sheetData>
@@ -2254,24 +2577,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="12" customHeight="1">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="24"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="26"/>
     </row>
     <row r="2" spans="1:6" ht="12" customHeight="1">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="27" t="s">
         <v>87</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
@@ -2411,7 +2734,7 @@
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="29" t="s">
+      <c r="A11" s="8" t="s">
         <v>264</v>
       </c>
       <c r="B11" s="19">
@@ -2427,24 +2750,24 @@
       <c r="E11" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="F11" s="28" t="s">
+      <c r="F11" s="9" t="s">
         <v>269</v>
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="29" t="s">
+      <c r="A12" s="8" t="s">
         <v>287</v>
       </c>
       <c r="B12" s="19">
         <f>B11*B33</f>
         <v>2303240.7407407407</v>
       </c>
-      <c r="C12" s="30" t="s">
+      <c r="C12" s="4" t="s">
         <v>119</v>
       </c>
       <c r="D12" s="4"/>
-      <c r="E12" s="30"/>
-      <c r="F12" s="28" t="s">
+      <c r="E12" s="4"/>
+      <c r="F12" s="9" t="s">
         <v>269</v>
       </c>
     </row>
@@ -2499,8 +2822,8 @@
       <c r="C16" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="D16" s="30"/>
-      <c r="E16" s="30"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
       <c r="F16" s="9"/>
     </row>
     <row r="17" spans="1:6" ht="28">
@@ -2586,7 +2909,7 @@
       </c>
     </row>
     <row r="21" spans="1:6" ht="28">
-      <c r="A21" s="29" t="s">
+      <c r="A21" s="8" t="s">
         <v>273</v>
       </c>
       <c r="B21" s="19">
@@ -2602,12 +2925,12 @@
       <c r="E21" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="F21" s="28" t="s">
+      <c r="F21" s="9" t="s">
         <v>269</v>
       </c>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" s="29" t="s">
+      <c r="A22" s="8" t="s">
         <v>286</v>
       </c>
       <c r="B22" s="19">
@@ -2620,7 +2943,7 @@
       <c r="E22" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="F22" s="28" t="s">
+      <c r="F22" s="9" t="s">
         <v>269</v>
       </c>
     </row>
@@ -2671,7 +2994,7 @@
       </c>
     </row>
     <row r="31" spans="1:6">
-      <c r="A31" s="27" t="s">
+      <c r="A31" s="4" t="s">
         <v>280</v>
       </c>
       <c r="B31">
@@ -2688,7 +3011,7 @@
       </c>
     </row>
     <row r="32" spans="1:6">
-      <c r="A32" s="27" t="s">
+      <c r="A32" s="4" t="s">
         <v>282</v>
       </c>
       <c r="B32">
@@ -2705,7 +3028,7 @@
       </c>
     </row>
     <row r="33" spans="1:3">
-      <c r="A33" s="27" t="s">
+      <c r="A33" s="4" t="s">
         <v>280</v>
       </c>
       <c r="B33">
@@ -2717,7 +3040,7 @@
       </c>
     </row>
     <row r="34" spans="1:3">
-      <c r="A34" s="27" t="s">
+      <c r="A34" s="4" t="s">
         <v>282</v>
       </c>
       <c r="B34">
@@ -2738,6 +3061,476 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF20DE3F-1803-4018-8B40-C6B40DCE81E4}">
+  <dimension ref="A1:F33"/>
+  <sheetFormatPr defaultRowHeight="14"/>
+  <cols>
+    <col min="1" max="1" width="28.75" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="4" max="4" width="27.5" customWidth="1"/>
+    <col min="5" max="5" width="10.6640625" customWidth="1"/>
+    <col min="6" max="6" width="35" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="24" customHeight="1">
+      <c r="A1" s="24" t="s">
+        <v>306</v>
+      </c>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="26"/>
+    </row>
+    <row r="2" spans="1:6" ht="12" customHeight="1">
+      <c r="A2" s="27" t="s">
+        <v>307</v>
+      </c>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="28">
+      <c r="A5" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>313</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>304</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>310</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="28">
+      <c r="A6" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="B6" s="19">
+        <v>5</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>314</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="F6" s="7" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="42">
+      <c r="A7" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="B7" s="19">
+        <v>2</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="E7" s="4"/>
+      <c r="F7" s="7" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="42">
+      <c r="A8" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="B8" s="31">
+        <f>B6/$B$29/$B$32</f>
+        <v>2.512562814070352E-4</v>
+      </c>
+      <c r="C8" s="30" t="s">
+        <v>317</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>314</v>
+      </c>
+      <c r="E8" s="4"/>
+      <c r="F8" s="9"/>
+    </row>
+    <row r="9" spans="1:6" ht="42">
+      <c r="A9" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="B9" s="31">
+        <f>B7/$B$29/$B$32</f>
+        <v>1.0050251256281407E-4</v>
+      </c>
+      <c r="C9" s="30" t="s">
+        <v>317</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="E9" s="4"/>
+      <c r="F9" s="9"/>
+    </row>
+    <row r="10" spans="1:6" ht="42">
+      <c r="A10" s="8" t="s">
+        <v>323</v>
+      </c>
+      <c r="B10" s="22">
+        <f>$B$9*Parameters!C29</f>
+        <v>1.7085427135678392E-2</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="F10" s="9"/>
+    </row>
+    <row r="11" spans="1:6" ht="42">
+      <c r="A11" s="8" t="s">
+        <v>325</v>
+      </c>
+      <c r="B11" s="22">
+        <f>$B$9*Parameters!C30</f>
+        <v>1.0552763819095477E-2</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="F11" s="12"/>
+    </row>
+    <row r="12" spans="1:6" ht="42">
+      <c r="A12" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="B12" s="22">
+        <f>$B$8*Parameters!C31</f>
+        <v>1.6331658291457288E-2</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="F12" s="9"/>
+    </row>
+    <row r="13" spans="1:6" ht="42">
+      <c r="A13" s="8" t="s">
+        <v>328</v>
+      </c>
+      <c r="B13" s="22">
+        <f>$B$8*Parameters!C29</f>
+        <v>4.2713567839195984E-2</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="F13" s="9"/>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="28">
+      <c r="A16" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="B16" s="13">
+        <v>0.7</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>310</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="42">
+      <c r="A17" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="B17" s="31">
+        <f>B16/$B$29/$B$33</f>
+        <v>3.111111111111111E-5</v>
+      </c>
+      <c r="C17" s="30" t="s">
+        <v>333</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="E17" s="4"/>
+      <c r="F17" s="9"/>
+    </row>
+    <row r="18" spans="1:6" ht="28">
+      <c r="A18" s="8" t="s">
+        <v>323</v>
+      </c>
+      <c r="B18" s="22">
+        <f>$B$17*Parameters!C29</f>
+        <v>5.288888888888889E-3</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="28">
+      <c r="A19" s="8" t="s">
+        <v>325</v>
+      </c>
+      <c r="B19" s="22">
+        <f>$B$17*Parameters!C30</f>
+        <v>3.2666666666666664E-3</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D19" s="11" t="s">
+        <v>267</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="28">
+      <c r="A20" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="B20" s="22">
+        <f>$B$17*Parameters!C31</f>
+        <v>2.0222222222222221E-3</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="28">
+      <c r="A21" s="8" t="s">
+        <v>328</v>
+      </c>
+      <c r="B21" s="22">
+        <f>$B$17*Parameters!C29</f>
+        <v>5.288888888888889E-3</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="E21" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="98">
+      <c r="A24" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="98">
+      <c r="A25" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="70">
+      <c r="A26" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" s="8" t="s">
+        <v>275</v>
+      </c>
+      <c r="B29" s="14">
+        <v>3600</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="B30">
+        <v>19.899999999999999</v>
+      </c>
+      <c r="C30" t="s">
+        <v>278</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="E30" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="B31">
+        <v>22.5</v>
+      </c>
+      <c r="C31" t="s">
+        <v>278</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="E31" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="B32">
+        <f>B30/$B$29*1000</f>
+        <v>5.5277777777777777</v>
+      </c>
+      <c r="C32" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="B33">
+        <f>B31/$B$29*1000</f>
+        <v>6.25</v>
+      </c>
+      <c r="C33" t="s">
+        <v>285</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G41"/>
   <sheetFormatPr defaultRowHeight="14"/>
@@ -2752,26 +3545,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18" customHeight="1">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="24"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="26"/>
     </row>
     <row r="2" spans="1:7" ht="12" customHeight="1">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="27" t="s">
         <v>115</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="1" t="s">
@@ -2837,7 +3630,7 @@
       <c r="A7" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="B7" s="26">
+      <c r="B7" s="22">
         <v>0.20100000000000001</v>
       </c>
       <c r="C7" s="4" t="s">
@@ -2889,7 +3682,7 @@
       <c r="E9" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="F9" s="27" t="s">
+      <c r="F9" s="4" t="s">
         <v>242</v>
       </c>
     </row>
@@ -3012,7 +3805,7 @@
       <c r="E16" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="F16" s="27" t="s">
+      <c r="F16" s="4" t="s">
         <v>242</v>
       </c>
     </row>
@@ -3196,7 +3989,7 @@
       <c r="E25" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="F25" s="27" t="s">
+      <c r="F25" s="4" t="s">
         <v>242</v>
       </c>
     </row>
@@ -3217,7 +4010,7 @@
       <c r="E26" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="F26" s="27" t="s">
+      <c r="F26" s="4" t="s">
         <v>242</v>
       </c>
     </row>
@@ -3238,7 +4031,7 @@
       <c r="E27" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="F27" s="27" t="s">
+      <c r="F27" s="4" t="s">
         <v>242</v>
       </c>
     </row>
@@ -3327,14 +4120,14 @@
       </c>
     </row>
     <row r="32" spans="1:6">
-      <c r="A32" s="30"/>
-      <c r="B32" s="32"/>
-      <c r="C32" s="30"/>
+      <c r="A32" s="4"/>
+      <c r="B32" s="19"/>
+      <c r="C32" s="4"/>
       <c r="D32" s="4"/>
-      <c r="E32" s="30"/>
-      <c r="F32" s="30"/>
-    </row>
-    <row r="34" spans="1:7" ht="28">
+      <c r="E32" s="4"/>
+      <c r="F32" s="4"/>
+    </row>
+    <row r="34" spans="1:7">
       <c r="A34" s="1" t="s">
         <v>148</v>
       </c>
@@ -3494,7 +4287,7 @@
       <c r="E41" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="F41" s="28" t="s">
+      <c r="F41" s="9" t="s">
         <v>261</v>
       </c>
     </row>
@@ -3507,7 +4300,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="14"/>
@@ -3523,28 +4316,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="12" customHeight="1">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="24" t="s">
         <v>162</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="24"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="26"/>
     </row>
     <row r="2" spans="1:8" ht="12" customHeight="1">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="27" t="s">
         <v>163</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="1" t="s">
@@ -3821,9 +4614,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="8.75" customWidth="1"/>
@@ -3834,22 +4627,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="12" customHeight="1">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="24" t="s">
         <v>197</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="24"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="26"/>
     </row>
     <row r="2" spans="1:5" ht="12" customHeight="1">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="27" t="s">
         <v>198</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
@@ -4002,6 +4795,14 @@
       </c>
       <c r="E12" s="12" t="s">
         <v>234</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="28" t="s">
+        <v>310</v>
+      </c>
+      <c r="B13" s="29" t="s">
+        <v>311</v>
       </c>
     </row>
   </sheetData>

</xml_diff>